<commit_message>
add test data and reports
</commit_message>
<xml_diff>
--- a/Data/Search_data.xlsx
+++ b/Data/Search_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\test_TL\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8039969-5806-4C30-A7FD-3E9E7F568774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D537FE7-DFEC-451B-83CF-03EBB7E7942B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2788D3C6-25EF-4D4A-9316-40D19310986B}"/>
   </bookViews>
@@ -55,7 +55,7 @@
     <t>!@#$%</t>
   </si>
   <si>
-    <t>CÓ 131 KẾT QUẢ TÌM KIẾM PHÙ HỢP</t>
+    <t>CÓ 130 KẾT QUẢ TÌM KIẾM PHÙ HỢP</t>
   </si>
 </sst>
 </file>

</xml_diff>